<commit_message>
review1 in sync with newrdk9arch and b align
</commit_message>
<xml_diff>
--- a/video/rdk9/Southbound-apis.xlsx
+++ b/video/rdk9/Southbound-apis.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ldhana149\RDKE-components-registry\RDK9\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ldhana149\rdk-core-specs\video\rdk9\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{24CC38ED-05A7-45FB-A349-32D211A3847E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4AFAEE17-1E5E-496F-A08B-56CE2FBEDBBF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{FAF072B6-16C5-45D0-A7E0-DB98C7C84CF4}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="28" uniqueCount="23">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="36" uniqueCount="26">
   <si>
     <t>HAL interface</t>
   </si>
@@ -65,9 +65,6 @@
     <t>https://github.com/rdkcentral/rdk-halif-rmf_audio_capture</t>
   </si>
   <si>
-    <t>https://github.com/rdkcentral/control</t>
-  </si>
-  <si>
     <t>Power Manager HAL</t>
   </si>
   <si>
@@ -89,18 +86,9 @@
     <t>systemaudioplatform HAL</t>
   </si>
   <si>
-    <t>Crypto HAL</t>
-  </si>
-  <si>
     <t>Bluetooth HAL</t>
   </si>
   <si>
-    <t>Sysint HAL</t>
-  </si>
-  <si>
-    <t>Westeros SOC HAL</t>
-  </si>
-  <si>
     <t>Graphics &amp; Matrix HAL</t>
   </si>
   <si>
@@ -108,6 +96,27 @@
   </si>
   <si>
     <t>develop</t>
+  </si>
+  <si>
+    <t>Westeros Graphics HAL</t>
+  </si>
+  <si>
+    <t>Westeros Sink HAL</t>
+  </si>
+  <si>
+    <t>https://github.com/rdkcentral/rdk-halif-systemaudioplatform</t>
+  </si>
+  <si>
+    <t>https://github.com/rdkcentral/rdk-halif-irdb</t>
+  </si>
+  <si>
+    <t>https://github.com/rdkcentral/bluetooth_vendor_document</t>
+  </si>
+  <si>
+    <t>https://github.com/rdkcentral/rdk-hpk-documentation/doc/Media_Pipeline</t>
+  </si>
+  <si>
+    <t>https://github.com/rdkcentral/rdk-halif-westeros-gl</t>
   </si>
 </sst>
 </file>
@@ -490,7 +499,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6CB4C54F-9F48-432F-BDFD-60E9A20D0936}">
-  <dimension ref="A1:C14"/>
+  <dimension ref="A1:C13"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="27.26953125" customWidth="1"/>
@@ -503,7 +512,7 @@
         <v>0</v>
       </c>
       <c r="B1" t="s">
-        <v>21</v>
+        <v>17</v>
       </c>
       <c r="C1" t="s">
         <v>1</v>
@@ -514,18 +523,18 @@
         <v>2</v>
       </c>
       <c r="B2" t="s">
-        <v>22</v>
-      </c>
-      <c r="C2" t="s">
+        <v>18</v>
+      </c>
+      <c r="C2" s="1" t="s">
         <v>3</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="B3" t="s">
-        <v>22</v>
+        <v>18</v>
       </c>
       <c r="C3" s="1" t="s">
         <v>4</v>
@@ -533,10 +542,10 @@
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="B4" t="s">
-        <v>22</v>
+        <v>18</v>
       </c>
       <c r="C4" s="1" t="s">
         <v>5</v>
@@ -544,10 +553,10 @@
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B5" t="s">
-        <v>22</v>
+        <v>18</v>
       </c>
       <c r="C5" s="1" t="s">
         <v>6</v>
@@ -555,10 +564,10 @@
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B6" t="s">
-        <v>22</v>
+        <v>18</v>
       </c>
       <c r="C6" s="1" t="s">
         <v>7</v>
@@ -566,48 +575,70 @@
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B7" t="s">
+        <v>18</v>
+      </c>
+      <c r="C7" s="1" t="s">
         <v>22</v>
-      </c>
-      <c r="C7" s="1" t="s">
-        <v>8</v>
       </c>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
-        <v>15</v>
+        <v>14</v>
+      </c>
+      <c r="B9" t="s">
+        <v>18</v>
+      </c>
+      <c r="C9" s="1" t="s">
+        <v>21</v>
       </c>
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
-        <v>16</v>
+        <v>15</v>
+      </c>
+      <c r="B10" t="s">
+        <v>18</v>
+      </c>
+      <c r="C10" s="1" t="s">
+        <v>23</v>
       </c>
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A11" t="s">
-        <v>17</v>
+        <v>20</v>
+      </c>
+      <c r="B11" t="s">
+        <v>18</v>
       </c>
     </row>
     <row r="12" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A12" t="s">
-        <v>18</v>
+        <v>19</v>
+      </c>
+      <c r="B12" t="s">
+        <v>18</v>
+      </c>
+      <c r="C12" s="1" t="s">
+        <v>25</v>
       </c>
     </row>
     <row r="13" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A13" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="14" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A14" t="s">
-        <v>20</v>
+        <v>16</v>
+      </c>
+      <c r="B13" t="s">
+        <v>18</v>
+      </c>
+      <c r="C13" s="1" t="s">
+        <v>24</v>
       </c>
     </row>
   </sheetData>
@@ -617,8 +648,13 @@
     <hyperlink ref="C5" r:id="rId3" xr:uid="{351C2C1E-4F06-4E38-8ED1-DD9926123F3C}"/>
     <hyperlink ref="C6" r:id="rId4" xr:uid="{DC5C67D3-B02E-44F6-935F-5396FC9227AC}"/>
     <hyperlink ref="C7" r:id="rId5" xr:uid="{5FA93519-2A90-494F-A1B7-2A0C1410D901}"/>
+    <hyperlink ref="C9" r:id="rId6" xr:uid="{A4DAF6AC-9CB6-4654-A38E-5CB5AF737908}"/>
+    <hyperlink ref="C10" r:id="rId7" xr:uid="{5FC485AD-F7AE-40D0-BDA6-150D3AC3EB2C}"/>
+    <hyperlink ref="C13" r:id="rId8" xr:uid="{0B400734-6F84-4B61-A991-083E2FDFBC1F}"/>
+    <hyperlink ref="C12" r:id="rId9" xr:uid="{7EA91A82-47DF-4FEF-88F9-046B7DD2272A}"/>
+    <hyperlink ref="C2" r:id="rId10" xr:uid="{A50A4D0D-315C-4B62-A71B-409A832F83DD}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" r:id="rId6"/>
+  <pageSetup orientation="portrait" r:id="rId11"/>
 </worksheet>
 </file>
</xml_diff>